<commit_message>
update only project C#
</commit_message>
<xml_diff>
--- a/15-11-2025 HMS-TAX/HMS-TAX/bin/Debug/Reports/rpt_customer_info.xlsx
+++ b/15-11-2025 HMS-TAX/HMS-TAX/bin/Debug/Reports/rpt_customer_info.xlsx
@@ -1,23 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JoinCoder\OneDrive\Desktop\CLINIC\CLINIC\bin\Debug\Reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_Dev\HMS-TAX\HMS-TAX\bin\Debug\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202D899B-8E32-43A1-BC95-A331EF056948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{881B3445-3BD5-48AC-BEAB-3DDF33B07567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Customer Info" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="125725"/>
 </workbook>
 </file>
 
@@ -33,38 +31,32 @@
     <t>Customer information</t>
   </si>
   <si>
-    <t>Gender</t>
-  </si>
-  <si>
     <t>Phone</t>
   </si>
   <si>
-    <t>Address</t>
-  </si>
-  <si>
     <t xml:space="preserve">Name </t>
   </si>
   <si>
     <t>Cus.ID</t>
+  </si>
+  <si>
+    <t>Remark</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <sz val="20"/>
@@ -74,26 +66,33 @@
     </font>
     <font>
       <b/>
-      <i/>
-      <sz val="12"/>
-      <color rgb="FF002060"/>
-      <name val="Times New Roman"/>
+      <sz val="20"/>
+      <color theme="3" tint="0.39997558519241921"/>
+      <name val="Cooper Black"/>
       <family val="1"/>
     </font>
     <font>
-      <b/>
-      <sz val="20"/>
+      <i/>
+      <sz val="11"/>
       <color rgb="FF002060"/>
-      <name val="Times New Roman"/>
+      <name val="CooperFiveOpti Black"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF002060"/>
+      <name val="Cooper Black"/>
       <family val="1"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF002060"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <color theme="1"/>
+      <name val="Khmer OS Battambang"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="3" tint="0.39997558519241921"/>
+      <name val="Khmer OS Battambang"/>
     </font>
   </fonts>
   <fills count="3">
@@ -105,7 +104,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -137,10 +136,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -149,29 +147,35 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -191,10 +195,65 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>485775</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8519FC69-1858-690C-5D11-78504999001B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="257175" y="0"/>
+          <a:ext cx="657225" cy="657225"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -232,9 +291,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -267,26 +326,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -319,26 +361,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -512,79 +537,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.6640625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="5.33203125" style="7" customWidth="1"/>
-    <col min="3" max="3" width="12" style="7" customWidth="1"/>
-    <col min="4" max="4" width="20.77734375" style="7" customWidth="1"/>
-    <col min="5" max="5" width="12" style="7" customWidth="1"/>
-    <col min="6" max="6" width="18" style="7" customWidth="1"/>
-    <col min="7" max="7" width="34.33203125" style="8" customWidth="1"/>
-    <col min="8" max="8" width="16.44140625" style="4" customWidth="1"/>
-    <col min="9" max="9" width="16.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="1.7109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" style="12" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" style="11" customWidth="1"/>
+    <col min="4" max="4" width="22.5703125" style="11" customWidth="1"/>
+    <col min="5" max="5" width="18" style="11" customWidth="1"/>
+    <col min="6" max="6" width="34.28515625" style="11" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" style="13" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" customFormat="1" ht="8.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+    <row r="1" spans="1:8" ht="8.4499999999999993" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1"/>
+      <c r="B1" s="6"/>
+      <c r="C1"/>
+      <c r="D1"/>
+      <c r="E1"/>
+      <c r="F1"/>
+      <c r="G1" s="6"/>
+      <c r="H1"/>
     </row>
-    <row r="2" spans="2:9" customFormat="1" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="10" t="s">
+    <row r="2" spans="1:8" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2"/>
+      <c r="B2" s="6"/>
+      <c r="C2"/>
+      <c r="D2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
       <c r="G2" s="5"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="2:9" customFormat="1" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
+    <row r="3" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3"/>
+      <c r="B3" s="6"/>
+      <c r="C3"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
       <c r="G3" s="5"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="H3" s="1"/>
     </row>
-    <row r="4" spans="2:9" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="11"/>
-      <c r="C4" s="12" t="s">
+    <row r="4" spans="1:8" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="10">
         <v>42285</v>
       </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="E4" s="2"/>
+      <c r="F4"/>
+      <c r="G4" s="6"/>
+      <c r="H4"/>
     </row>
-    <row r="5" spans="2:9" customFormat="1" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="9" t="s">
+    <row r="5" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5"/>
+      <c r="B5" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>5</v>
-      </c>
+      <c r="H5"/>
+    </row>
+    <row r="11" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F11" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -592,23 +627,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>